<commit_message>
Drop product_description column (keep unit): remove from Suppliers + SupplierMetrics zod schemas, route mapping, scores.IDENTITY_COLS, python.ts types, both sample sheets, and Supplier.productDescription (migration). unit retained everywhere. product_description was read by nothing (validated-only dead column). Import output byte-identical for staying columns.
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/procurement_data_raw.xlsx
+++ b/data/raw/procurement_data_raw.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,16 +451,6 @@
           <t>category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>product_description</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>tier</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -483,16 +473,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Komatsu authorized dealer (haul trucks, dozers, excavators)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,16 +495,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Caterpillar dealer for Indonesia</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -547,16 +517,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Hitachi construction machinery distributor</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -579,16 +539,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Underground mining equipment, crushers, drills</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -611,16 +561,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Mining excavators, mobile cranes</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -643,16 +583,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Drilling rigs, rock excavation equipment</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -675,16 +605,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Doosan heavy equipment dealer</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -707,16 +627,6 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Articulated haulers, wheel loaders</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -739,16 +649,6 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OTR mining tires (radial and bias)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -771,16 +671,6 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Mining and industrial OTR tires</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -803,16 +693,6 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Industrial and OTR tires</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -835,16 +715,6 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Specialty industrial tires</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -867,16 +737,6 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Local industrial tires</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -899,16 +759,6 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>State-owned: explosives, blasting services</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -931,16 +781,6 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Ammonium nitrate, initiating systems</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -963,16 +803,6 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Commercial explosives manufacturer</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -995,16 +825,6 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Industrial fuel and lubricants - HSD, B30, marine fuels</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1027,16 +847,6 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Industrial fuels, lubricants</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1059,16 +869,6 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Fuels and lubricants</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1091,16 +891,6 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Mobil Delvac heavy-duty lubricants</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1123,16 +913,6 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Industrial and mining lubricants</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1155,16 +935,6 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Lubricants and specialty fluids</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1187,16 +957,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Mining contracting, overburden removal</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1219,16 +979,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Coal mining contractor</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1251,16 +1001,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Mining and EPC contractor</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1283,16 +1023,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Mining contracting services</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1315,16 +1045,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Mining contracting, equipment rental</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1347,16 +1067,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Mining services contractor</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1379,16 +1089,6 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Mining contractor (smaller scale)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1411,16 +1111,6 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Drilling rigs, compressors</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1443,16 +1133,6 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Hydraulic rock drills</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1475,16 +1155,6 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Heavy drilling equipment</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1507,16 +1177,6 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Drill bits, core barrels, drilling tools</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1539,16 +1199,6 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Drill bits, rods, sleeves</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1571,16 +1221,6 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Drilling consumables and supplies</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1603,16 +1243,6 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Wear parts, GET (ground engaging tools)</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1635,16 +1265,6 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Engineered wear parts</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1667,16 +1287,6 @@
           <t>Conveyor &amp; Belt</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Steel cord conveyor belts, splice services</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1699,16 +1309,6 @@
           <t>Conveyor &amp; Belt</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Conveyor belts and components</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1731,16 +1331,6 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>PPE, respirators, safety equipment</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1763,16 +1353,6 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Industrial PPE, gas detection</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1795,16 +1375,6 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Local PPE distribution</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1827,16 +1397,6 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Electrical systems, automation</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1859,16 +1419,6 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Power distribution equipment</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1891,16 +1441,6 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Industrial automation, drives</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1923,16 +1463,6 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Steel plates, structural steel</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1955,16 +1485,6 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Steel products</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1987,16 +1507,6 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Steel fabrication</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2019,16 +1529,6 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Local fabrication services</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2051,16 +1551,6 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Welding and fabrication</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2083,16 +1573,6 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Heavy hauling, logistics services</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2115,16 +1595,6 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Coal shipping services</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2147,16 +1617,6 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Land transportation</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2179,16 +1639,6 @@
           <t>Spare Parts &amp; Components</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Genuine spare parts distribution</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2209,16 +1659,6 @@
       <c r="D56" t="inlineStr">
         <is>
           <t>Spare Parts &amp; Components</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Aftermarket spare parts</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Standard</t>
         </is>
       </c>
     </row>
@@ -58643,7 +58083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -58669,70 +58109,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>product_description</t>
+          <t>defect_rate_pct</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>tier</t>
+          <t>complaint_count_annual</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>total_spend_usd</t>
+          <t>rfx_response_rate_pct</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>num_pos</t>
+          <t>avg_response_time_days</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>avg_po_value_usd</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>avg_lead_time_days</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>avg_cycle_time_days</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>on_time_delivery_pct</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>three_way_match_pct</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>defect_rate_pct</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>complaint_count_annual</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>rfx_response_rate_pct</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>avg_response_time_days</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>single_source_risk</t>
         </is>
@@ -58759,50 +58154,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Komatsu authorized dealer (haul trucks, dozers, excavators)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E2" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>64243644.56</v>
+        <v>94.72</v>
       </c>
       <c r="H2" t="n">
-        <v>26</v>
+        <v>1.97</v>
       </c>
       <c r="I2" t="n">
-        <v>2470909.41</v>
-      </c>
-      <c r="J2" t="n">
-        <v>9.92</v>
-      </c>
-      <c r="K2" t="n">
-        <v>28.73</v>
-      </c>
-      <c r="L2" t="n">
-        <v>88.45999999999999</v>
-      </c>
-      <c r="M2" t="n">
-        <v>84.62</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>94.72</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>1.97</v>
-      </c>
-      <c r="R2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58827,50 +58191,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Caterpillar dealer for Indonesia</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>74982592.87</v>
+        <v>97.61</v>
       </c>
       <c r="H3" t="n">
-        <v>28</v>
+        <v>1.3</v>
       </c>
       <c r="I3" t="n">
-        <v>2677949.75</v>
-      </c>
-      <c r="J3" t="n">
-        <v>9.539999999999999</v>
-      </c>
-      <c r="K3" t="n">
-        <v>30.21</v>
-      </c>
-      <c r="L3" t="n">
-        <v>92.86</v>
-      </c>
-      <c r="M3" t="n">
-        <v>78.56999999999999</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>97.61</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58895,50 +58228,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Hitachi construction machinery distributor</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E4" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>78575964.45</v>
+        <v>82.02</v>
       </c>
       <c r="H4" t="n">
-        <v>31</v>
+        <v>1.01</v>
       </c>
       <c r="I4" t="n">
-        <v>2534708.53</v>
-      </c>
-      <c r="J4" t="n">
-        <v>11.39</v>
-      </c>
-      <c r="K4" t="n">
-        <v>33.29</v>
-      </c>
-      <c r="L4" t="n">
-        <v>83.87</v>
-      </c>
-      <c r="M4" t="n">
-        <v>67.73999999999999</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>82.02</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="R4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58963,50 +58265,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Underground mining equipment, crushers, drills</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E5" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>71381757.84</v>
+        <v>98.41</v>
       </c>
       <c r="H5" t="n">
-        <v>26</v>
+        <v>1.13</v>
       </c>
       <c r="I5" t="n">
-        <v>2745452.22</v>
-      </c>
-      <c r="J5" t="n">
-        <v>22.12</v>
-      </c>
-      <c r="K5" t="n">
-        <v>43.73</v>
-      </c>
-      <c r="L5" t="n">
-        <v>88.45999999999999</v>
-      </c>
-      <c r="M5" t="n">
-        <v>88.45999999999999</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="O5" t="n">
-        <v>2</v>
-      </c>
-      <c r="P5" t="n">
-        <v>98.41</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="R5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59031,50 +58302,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Mining excavators, mobile cranes</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E6" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>62091581.09</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="H6" t="n">
-        <v>26</v>
+        <v>1.3</v>
       </c>
       <c r="I6" t="n">
-        <v>2388137.73</v>
-      </c>
-      <c r="J6" t="n">
-        <v>21.58</v>
-      </c>
-      <c r="K6" t="n">
-        <v>46.46</v>
-      </c>
-      <c r="L6" t="n">
-        <v>80.77</v>
-      </c>
-      <c r="M6" t="n">
-        <v>69.23</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="O6" t="n">
-        <v>3</v>
-      </c>
-      <c r="P6" t="n">
-        <v>93.70999999999999</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="R6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59099,50 +58339,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Drilling rigs, rock excavation equipment</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E7" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>38980562.92</v>
+        <v>92.22</v>
       </c>
       <c r="H7" t="n">
-        <v>15</v>
+        <v>1.48</v>
       </c>
       <c r="I7" t="n">
-        <v>2598704.19</v>
-      </c>
-      <c r="J7" t="n">
-        <v>21.07</v>
-      </c>
-      <c r="K7" t="n">
-        <v>40.47</v>
-      </c>
-      <c r="L7" t="n">
-        <v>93.33</v>
-      </c>
-      <c r="M7" t="n">
-        <v>73.33</v>
-      </c>
-      <c r="N7" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="O7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" t="n">
-        <v>92.22</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="R7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59167,50 +58376,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Doosan heavy equipment dealer</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E8" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="F8" t="n">
+        <v>7</v>
       </c>
       <c r="G8" t="n">
-        <v>19555684.62</v>
+        <v>78.98</v>
       </c>
       <c r="H8" t="n">
-        <v>7</v>
+        <v>2.4</v>
       </c>
       <c r="I8" t="n">
-        <v>2793669.23</v>
-      </c>
-      <c r="J8" t="n">
-        <v>10.29</v>
-      </c>
-      <c r="K8" t="n">
-        <v>30.29</v>
-      </c>
-      <c r="L8" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="M8" t="n">
-        <v>100</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="O8" t="n">
-        <v>7</v>
-      </c>
-      <c r="P8" t="n">
-        <v>78.98</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="R8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59235,50 +58413,19 @@
           <t>Heavy Equipment OEM</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Articulated haulers, wheel loaders</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E9" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>23917188.18</v>
+        <v>83.43000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>12</v>
+        <v>5.44</v>
       </c>
       <c r="I9" t="n">
-        <v>1993099.02</v>
-      </c>
-      <c r="J9" t="n">
-        <v>22.33</v>
-      </c>
-      <c r="K9" t="n">
-        <v>47.17</v>
-      </c>
-      <c r="L9" t="n">
-        <v>91.67</v>
-      </c>
-      <c r="M9" t="n">
-        <v>91.67</v>
-      </c>
-      <c r="N9" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="O9" t="n">
-        <v>2</v>
-      </c>
-      <c r="P9" t="n">
-        <v>83.43000000000001</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>5.44</v>
-      </c>
-      <c r="R9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59303,50 +58450,19 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OTR mining tires (radial and bias)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E10" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>12062506.55</v>
+        <v>88.48999999999999</v>
       </c>
       <c r="H10" t="n">
-        <v>22</v>
+        <v>1.9</v>
       </c>
       <c r="I10" t="n">
-        <v>548295.75</v>
-      </c>
-      <c r="J10" t="n">
-        <v>9.68</v>
-      </c>
-      <c r="K10" t="n">
-        <v>31.95</v>
-      </c>
-      <c r="L10" t="n">
-        <v>95.45</v>
-      </c>
-      <c r="M10" t="n">
-        <v>63.64</v>
-      </c>
-      <c r="N10" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O10" t="n">
-        <v>2</v>
-      </c>
-      <c r="P10" t="n">
-        <v>88.48999999999999</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="R10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59371,50 +58487,19 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Mining and industrial OTR tires</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>13198046.79</v>
+        <v>92.70999999999999</v>
       </c>
       <c r="H11" t="n">
-        <v>23</v>
+        <v>0.99</v>
       </c>
       <c r="I11" t="n">
-        <v>573828.12</v>
-      </c>
-      <c r="J11" t="n">
-        <v>22.09</v>
-      </c>
-      <c r="K11" t="n">
-        <v>46.17</v>
-      </c>
-      <c r="L11" t="n">
-        <v>91.3</v>
-      </c>
-      <c r="M11" t="n">
-        <v>73.91</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1</v>
-      </c>
-      <c r="P11" t="n">
-        <v>92.70999999999999</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="R11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59439,50 +58524,19 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Industrial and OTR tires</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E12" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>4531404.63</v>
+        <v>93.68000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>8</v>
+        <v>1.8</v>
       </c>
       <c r="I12" t="n">
-        <v>566425.58</v>
-      </c>
-      <c r="J12" t="n">
-        <v>9.380000000000001</v>
-      </c>
-      <c r="K12" t="n">
-        <v>30.88</v>
-      </c>
-      <c r="L12" t="n">
-        <v>100</v>
-      </c>
-      <c r="M12" t="n">
-        <v>75</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="O12" t="n">
-        <v>4</v>
-      </c>
-      <c r="P12" t="n">
-        <v>93.68000000000001</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="R12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59507,50 +58561,19 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Specialty industrial tires</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E13" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>3170262.67</v>
+        <v>92.48999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>9</v>
+        <v>4.37</v>
       </c>
       <c r="I13" t="n">
-        <v>352251.41</v>
-      </c>
-      <c r="J13" t="n">
-        <v>24</v>
-      </c>
-      <c r="K13" t="n">
-        <v>44.33</v>
-      </c>
-      <c r="L13" t="n">
-        <v>88.89</v>
-      </c>
-      <c r="M13" t="n">
-        <v>77.78</v>
-      </c>
-      <c r="N13" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="O13" t="n">
-        <v>3</v>
-      </c>
-      <c r="P13" t="n">
-        <v>92.48999999999999</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>4.37</v>
-      </c>
-      <c r="R13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -59575,50 +58598,19 @@
           <t>Tires</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Local industrial tires</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E14" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>2449235.35</v>
+        <v>75.2</v>
       </c>
       <c r="H14" t="n">
-        <v>3</v>
+        <v>7.07</v>
       </c>
       <c r="I14" t="n">
-        <v>816411.78</v>
-      </c>
-      <c r="J14" t="n">
-        <v>9</v>
-      </c>
-      <c r="K14" t="n">
-        <v>38</v>
-      </c>
-      <c r="L14" t="n">
-        <v>100</v>
-      </c>
-      <c r="M14" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="N14" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="O14" t="n">
-        <v>4</v>
-      </c>
-      <c r="P14" t="n">
-        <v>75.2</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="R14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59643,50 +58635,19 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>State-owned: explosives, blasting services</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E15" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>1849312.7</v>
+        <v>96.39</v>
       </c>
       <c r="H15" t="n">
-        <v>29</v>
+        <v>1.26</v>
       </c>
       <c r="I15" t="n">
-        <v>63769.4</v>
-      </c>
-      <c r="J15" t="n">
-        <v>8.93</v>
-      </c>
-      <c r="K15" t="n">
-        <v>35.66</v>
-      </c>
-      <c r="L15" t="n">
-        <v>100</v>
-      </c>
-      <c r="M15" t="n">
-        <v>55.17</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="O15" t="n">
-        <v>1</v>
-      </c>
-      <c r="P15" t="n">
-        <v>96.39</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="R15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -59711,50 +58672,19 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Ammonium nitrate, initiating systems</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E16" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>1004267.55</v>
+        <v>90.84</v>
       </c>
       <c r="H16" t="n">
-        <v>15</v>
+        <v>1.13</v>
       </c>
       <c r="I16" t="n">
-        <v>66951.17</v>
-      </c>
-      <c r="J16" t="n">
-        <v>21.47</v>
-      </c>
-      <c r="K16" t="n">
-        <v>43.07</v>
-      </c>
-      <c r="L16" t="n">
-        <v>93.33</v>
-      </c>
-      <c r="M16" t="n">
-        <v>73.33</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0.92</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="n">
-        <v>90.84</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="R16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59779,50 +58709,19 @@
           <t>Explosives</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Commercial explosives manufacturer</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E17" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
       </c>
       <c r="G17" t="n">
-        <v>481426.23</v>
+        <v>54.71</v>
       </c>
       <c r="H17" t="n">
-        <v>7</v>
+        <v>4.35</v>
       </c>
       <c r="I17" t="n">
-        <v>68775.17999999999</v>
-      </c>
-      <c r="J17" t="n">
-        <v>12</v>
-      </c>
-      <c r="K17" t="n">
-        <v>33.14</v>
-      </c>
-      <c r="L17" t="n">
-        <v>71.43000000000001</v>
-      </c>
-      <c r="M17" t="n">
-        <v>42.86</v>
-      </c>
-      <c r="N17" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="O17" t="n">
-        <v>2</v>
-      </c>
-      <c r="P17" t="n">
-        <v>54.71</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="R17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59847,50 +58746,19 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Industrial fuel and lubricants - HSD, B30, marine fuels</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E18" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>1244834.71</v>
+        <v>96.04000000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>16</v>
+        <v>0.68</v>
       </c>
       <c r="I18" t="n">
-        <v>77802.17</v>
-      </c>
-      <c r="J18" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="K18" t="n">
-        <v>30.75</v>
-      </c>
-      <c r="L18" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="M18" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="N18" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="n">
-        <v>96.04000000000001</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="R18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -59915,50 +58783,19 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Industrial fuels, lubricants</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E19" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>1343244.13</v>
+        <v>83.56</v>
       </c>
       <c r="H19" t="n">
-        <v>15</v>
+        <v>2.98</v>
       </c>
       <c r="I19" t="n">
-        <v>89549.61</v>
-      </c>
-      <c r="J19" t="n">
-        <v>11.73</v>
-      </c>
-      <c r="K19" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="L19" t="n">
-        <v>80</v>
-      </c>
-      <c r="M19" t="n">
-        <v>53.33</v>
-      </c>
-      <c r="N19" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="O19" t="n">
-        <v>2</v>
-      </c>
-      <c r="P19" t="n">
-        <v>83.56</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="R19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -59983,50 +58820,19 @@
           <t>Fuel</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Fuels and lubricants</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E20" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4</v>
       </c>
       <c r="G20" t="n">
-        <v>756423.73</v>
+        <v>72.22</v>
       </c>
       <c r="H20" t="n">
-        <v>10</v>
+        <v>1.24</v>
       </c>
       <c r="I20" t="n">
-        <v>75642.37</v>
-      </c>
-      <c r="J20" t="n">
-        <v>10</v>
-      </c>
-      <c r="K20" t="n">
-        <v>34.8</v>
-      </c>
-      <c r="L20" t="n">
-        <v>100</v>
-      </c>
-      <c r="M20" t="n">
-        <v>50</v>
-      </c>
-      <c r="N20" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="O20" t="n">
-        <v>4</v>
-      </c>
-      <c r="P20" t="n">
-        <v>72.22</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="R20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60051,50 +58857,19 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Mobil Delvac heavy-duty lubricants</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E21" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
       </c>
       <c r="G21" t="n">
-        <v>193547.22</v>
+        <v>71.88</v>
       </c>
       <c r="H21" t="n">
-        <v>13</v>
+        <v>0.8</v>
       </c>
       <c r="I21" t="n">
-        <v>14888.25</v>
-      </c>
-      <c r="J21" t="n">
-        <v>23.92</v>
-      </c>
-      <c r="K21" t="n">
-        <v>50.38</v>
-      </c>
-      <c r="L21" t="n">
-        <v>76.92</v>
-      </c>
-      <c r="M21" t="n">
-        <v>84.62</v>
-      </c>
-      <c r="N21" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="O21" t="n">
-        <v>2</v>
-      </c>
-      <c r="P21" t="n">
-        <v>71.88</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="R21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60119,50 +58894,19 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Industrial and mining lubricants</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E22" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F22" t="n">
+        <v>3</v>
       </c>
       <c r="G22" t="n">
-        <v>150367.68</v>
+        <v>65.76000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>8</v>
+        <v>2.2</v>
       </c>
       <c r="I22" t="n">
-        <v>18795.96</v>
-      </c>
-      <c r="J22" t="n">
-        <v>20.25</v>
-      </c>
-      <c r="K22" t="n">
-        <v>38</v>
-      </c>
-      <c r="L22" t="n">
-        <v>100</v>
-      </c>
-      <c r="M22" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="N22" t="n">
-        <v>2.49</v>
-      </c>
-      <c r="O22" t="n">
-        <v>3</v>
-      </c>
-      <c r="P22" t="n">
-        <v>65.76000000000001</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="R22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60187,50 +58931,19 @@
           <t>Lubricants</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Lubricants and specialty fluids</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E23" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>84768.56</v>
+        <v>65.45</v>
       </c>
       <c r="H23" t="n">
-        <v>4</v>
+        <v>5.91</v>
       </c>
       <c r="I23" t="n">
-        <v>21192.14</v>
-      </c>
-      <c r="J23" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="K23" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="L23" t="n">
-        <v>100</v>
-      </c>
-      <c r="M23" t="n">
-        <v>50</v>
-      </c>
-      <c r="N23" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="O23" t="n">
-        <v>2</v>
-      </c>
-      <c r="P23" t="n">
-        <v>65.45</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="R23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60255,50 +58968,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Mining contracting, overburden removal</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E24" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>7416638.44</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="H24" t="n">
-        <v>18</v>
+        <v>2.33</v>
       </c>
       <c r="I24" t="n">
-        <v>412035.47</v>
-      </c>
-      <c r="J24" t="n">
-        <v>10.22</v>
-      </c>
-      <c r="K24" t="n">
-        <v>33.44</v>
-      </c>
-      <c r="L24" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="M24" t="n">
-        <v>77.78</v>
-      </c>
-      <c r="N24" t="n">
-        <v>1.51</v>
-      </c>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="n">
-        <v>95.90000000000001</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="R24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60323,50 +59005,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Coal mining contractor</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E25" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3</v>
       </c>
       <c r="G25" t="n">
-        <v>11439210.32</v>
+        <v>94.29000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>26</v>
+        <v>1.49</v>
       </c>
       <c r="I25" t="n">
-        <v>439969.63</v>
-      </c>
-      <c r="J25" t="n">
-        <v>11.12</v>
-      </c>
-      <c r="K25" t="n">
-        <v>30.62</v>
-      </c>
-      <c r="L25" t="n">
-        <v>76.92</v>
-      </c>
-      <c r="M25" t="n">
-        <v>96.15000000000001</v>
-      </c>
-      <c r="N25" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="O25" t="n">
-        <v>3</v>
-      </c>
-      <c r="P25" t="n">
-        <v>94.29000000000001</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="R25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60391,50 +59042,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Mining and EPC contractor</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E26" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>15334098.15</v>
+        <v>94.73</v>
       </c>
       <c r="H26" t="n">
-        <v>31</v>
+        <v>3.37</v>
       </c>
       <c r="I26" t="n">
-        <v>494648.33</v>
-      </c>
-      <c r="J26" t="n">
-        <v>10.42</v>
-      </c>
-      <c r="K26" t="n">
-        <v>32.13</v>
-      </c>
-      <c r="L26" t="n">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="M26" t="n">
-        <v>54.84</v>
-      </c>
-      <c r="N26" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="O26" t="n">
-        <v>1</v>
-      </c>
-      <c r="P26" t="n">
-        <v>94.73</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>3.37</v>
-      </c>
-      <c r="R26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60459,50 +59079,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Mining contracting services</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E27" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
       </c>
       <c r="G27" t="n">
-        <v>3049603.07</v>
+        <v>57.36</v>
       </c>
       <c r="H27" t="n">
-        <v>6</v>
+        <v>2.42</v>
       </c>
       <c r="I27" t="n">
-        <v>508267.18</v>
-      </c>
-      <c r="J27" t="n">
-        <v>11.67</v>
-      </c>
-      <c r="K27" t="n">
-        <v>32.17</v>
-      </c>
-      <c r="L27" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="M27" t="n">
-        <v>100</v>
-      </c>
-      <c r="N27" t="n">
-        <v>2.01</v>
-      </c>
-      <c r="O27" t="n">
-        <v>3</v>
-      </c>
-      <c r="P27" t="n">
-        <v>57.36</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="R27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60527,50 +59116,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Mining contracting, equipment rental</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E28" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
       </c>
       <c r="G28" t="n">
-        <v>3128910.55</v>
+        <v>77.25</v>
       </c>
       <c r="H28" t="n">
-        <v>6</v>
+        <v>2.46</v>
       </c>
       <c r="I28" t="n">
-        <v>521485.09</v>
-      </c>
-      <c r="J28" t="n">
-        <v>9.33</v>
-      </c>
-      <c r="K28" t="n">
-        <v>27</v>
-      </c>
-      <c r="L28" t="n">
-        <v>100</v>
-      </c>
-      <c r="M28" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="N28" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="O28" t="n">
-        <v>5</v>
-      </c>
-      <c r="P28" t="n">
-        <v>77.25</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="R28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60595,50 +59153,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Mining services contractor</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E29" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F29" t="n">
+        <v>3</v>
       </c>
       <c r="G29" t="n">
-        <v>2123973.8</v>
+        <v>38.08</v>
       </c>
       <c r="H29" t="n">
-        <v>5</v>
+        <v>13.76</v>
       </c>
       <c r="I29" t="n">
-        <v>424794.76</v>
-      </c>
-      <c r="J29" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="K29" t="n">
-        <v>29.4</v>
-      </c>
-      <c r="L29" t="n">
-        <v>100</v>
-      </c>
-      <c r="M29" t="n">
-        <v>100</v>
-      </c>
-      <c r="N29" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="O29" t="n">
-        <v>3</v>
-      </c>
-      <c r="P29" t="n">
-        <v>38.08</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>13.76</v>
-      </c>
-      <c r="R29" t="n">
         <v>1</v>
       </c>
     </row>
@@ -60663,50 +59190,19 @@
           <t>Mining Contractor</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Mining contractor (smaller scale)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E30" t="n">
+        <v>6.45</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2</v>
       </c>
       <c r="G30" t="n">
-        <v>772871.11</v>
+        <v>31.58</v>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>4.64</v>
       </c>
       <c r="I30" t="n">
-        <v>386435.56</v>
-      </c>
-      <c r="J30" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="K30" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="L30" t="n">
-        <v>50</v>
-      </c>
-      <c r="M30" t="n">
-        <v>100</v>
-      </c>
-      <c r="N30" t="n">
-        <v>6.45</v>
-      </c>
-      <c r="O30" t="n">
-        <v>2</v>
-      </c>
-      <c r="P30" t="n">
-        <v>31.58</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="R30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60731,50 +59227,19 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Drilling rigs, compressors</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E31" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>25685617.23</v>
+        <v>96.91</v>
       </c>
       <c r="H31" t="n">
-        <v>22</v>
+        <v>1.96</v>
       </c>
       <c r="I31" t="n">
-        <v>1167528.06</v>
-      </c>
-      <c r="J31" t="n">
-        <v>23.23</v>
-      </c>
-      <c r="K31" t="n">
-        <v>46.41</v>
-      </c>
-      <c r="L31" t="n">
-        <v>77.27</v>
-      </c>
-      <c r="M31" t="n">
-        <v>81.81999999999999</v>
-      </c>
-      <c r="N31" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="O31" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" t="n">
-        <v>96.91</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>1.96</v>
-      </c>
-      <c r="R31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60799,50 +59264,19 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Hydraulic rock drills</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E32" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>12954752.64</v>
+        <v>82.36</v>
       </c>
       <c r="H32" t="n">
-        <v>9</v>
+        <v>3.42</v>
       </c>
       <c r="I32" t="n">
-        <v>1439416.96</v>
-      </c>
-      <c r="J32" t="n">
-        <v>23.44</v>
-      </c>
-      <c r="K32" t="n">
-        <v>43.67</v>
-      </c>
-      <c r="L32" t="n">
-        <v>100</v>
-      </c>
-      <c r="M32" t="n">
-        <v>77.78</v>
-      </c>
-      <c r="N32" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="O32" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" t="n">
-        <v>82.36</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>3.42</v>
-      </c>
-      <c r="R32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60867,50 +59301,19 @@
           <t>Drilling Equipment</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Heavy drilling equipment</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E33" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2</v>
       </c>
       <c r="G33" t="n">
-        <v>7223764.74</v>
+        <v>66.81999999999999</v>
       </c>
       <c r="H33" t="n">
-        <v>7</v>
+        <v>2.28</v>
       </c>
       <c r="I33" t="n">
-        <v>1031966.39</v>
-      </c>
-      <c r="J33" t="n">
-        <v>20.43</v>
-      </c>
-      <c r="K33" t="n">
-        <v>47.43</v>
-      </c>
-      <c r="L33" t="n">
-        <v>100</v>
-      </c>
-      <c r="M33" t="n">
-        <v>57.14</v>
-      </c>
-      <c r="N33" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="O33" t="n">
-        <v>2</v>
-      </c>
-      <c r="P33" t="n">
-        <v>66.81999999999999</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>2.28</v>
-      </c>
-      <c r="R33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -60935,50 +59338,19 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Drill bits, core barrels, drilling tools</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E34" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="F34" t="n">
+        <v>4</v>
       </c>
       <c r="G34" t="n">
-        <v>937340.15</v>
+        <v>63.46</v>
       </c>
       <c r="H34" t="n">
-        <v>10</v>
+        <v>1.66</v>
       </c>
       <c r="I34" t="n">
-        <v>93734.02</v>
-      </c>
-      <c r="J34" t="n">
-        <v>21.1</v>
-      </c>
-      <c r="K34" t="n">
-        <v>42.5</v>
-      </c>
-      <c r="L34" t="n">
-        <v>70</v>
-      </c>
-      <c r="M34" t="n">
-        <v>70</v>
-      </c>
-      <c r="N34" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="O34" t="n">
-        <v>4</v>
-      </c>
-      <c r="P34" t="n">
-        <v>63.46</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>1.66</v>
-      </c>
-      <c r="R34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61003,50 +59375,19 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Drill bits, rods, sleeves</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E35" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
       </c>
       <c r="G35" t="n">
-        <v>645561.46</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>8</v>
+        <v>3.26</v>
       </c>
       <c r="I35" t="n">
-        <v>80695.17999999999</v>
-      </c>
-      <c r="J35" t="n">
-        <v>20.88</v>
-      </c>
-      <c r="K35" t="n">
-        <v>40.38</v>
-      </c>
-      <c r="L35" t="n">
-        <v>75</v>
-      </c>
-      <c r="M35" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="N35" t="n">
-        <v>2.34</v>
-      </c>
-      <c r="O35" t="n">
-        <v>5</v>
-      </c>
-      <c r="P35" t="n">
-        <v>65.06999999999999</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="R35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61071,50 +59412,19 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Drilling consumables and supplies</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E36" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
       </c>
       <c r="G36" t="n">
-        <v>278036.11</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>4.07</v>
       </c>
       <c r="I36" t="n">
-        <v>139018.06</v>
-      </c>
-      <c r="J36" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="K36" t="n">
-        <v>39.5</v>
-      </c>
-      <c r="L36" t="n">
-        <v>100</v>
-      </c>
-      <c r="M36" t="n">
-        <v>50</v>
-      </c>
-      <c r="N36" t="n">
-        <v>6.18</v>
-      </c>
-      <c r="O36" t="n">
-        <v>5</v>
-      </c>
-      <c r="P36" t="n">
-        <v>82.93000000000001</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>4.07</v>
-      </c>
-      <c r="R36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61139,50 +59449,19 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Wear parts, GET (ground engaging tools)</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E37" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F37" t="n">
+        <v>3</v>
       </c>
       <c r="G37" t="n">
-        <v>1284272.73</v>
+        <v>62.08</v>
       </c>
       <c r="H37" t="n">
-        <v>15</v>
+        <v>6.92</v>
       </c>
       <c r="I37" t="n">
-        <v>85618.17999999999</v>
-      </c>
-      <c r="J37" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="K37" t="n">
-        <v>47.13</v>
-      </c>
-      <c r="L37" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="M37" t="n">
-        <v>86.67</v>
-      </c>
-      <c r="N37" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="O37" t="n">
-        <v>3</v>
-      </c>
-      <c r="P37" t="n">
-        <v>62.08</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>6.92</v>
-      </c>
-      <c r="R37" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61207,50 +59486,19 @@
           <t>Drilling Consumables</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Engineered wear parts</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E38" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
       </c>
       <c r="G38" t="n">
-        <v>180609.61</v>
+        <v>50.6</v>
       </c>
       <c r="H38" t="n">
-        <v>2</v>
+        <v>2.89</v>
       </c>
       <c r="I38" t="n">
-        <v>90304.8</v>
-      </c>
-      <c r="J38" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="K38" t="n">
-        <v>53.5</v>
-      </c>
-      <c r="L38" t="n">
-        <v>100</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="O38" t="n">
-        <v>5</v>
-      </c>
-      <c r="P38" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>2.89</v>
-      </c>
-      <c r="R38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61275,50 +59523,19 @@
           <t>Conveyor &amp; Belt</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Steel cord conveyor belts, splice services</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E39" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>408989.71</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>7</v>
+        <v>3.2</v>
       </c>
       <c r="I39" t="n">
-        <v>58427.1</v>
-      </c>
-      <c r="J39" t="n">
-        <v>21.71</v>
-      </c>
-      <c r="K39" t="n">
-        <v>40</v>
-      </c>
-      <c r="L39" t="n">
-        <v>100</v>
-      </c>
-      <c r="M39" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="N39" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="O39" t="n">
-        <v>2</v>
-      </c>
-      <c r="P39" t="n">
-        <v>69.31999999999999</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="R39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61343,50 +59560,19 @@
           <t>Conveyor &amp; Belt</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Conveyor belts and components</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E40" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
       </c>
       <c r="G40" t="n">
-        <v>138479.68</v>
+        <v>57.91</v>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>16.63</v>
       </c>
       <c r="I40" t="n">
-        <v>69239.84</v>
-      </c>
-      <c r="J40" t="n">
-        <v>20</v>
-      </c>
-      <c r="K40" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="L40" t="n">
-        <v>100</v>
-      </c>
-      <c r="M40" t="n">
-        <v>100</v>
-      </c>
-      <c r="N40" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="O40" t="n">
-        <v>5</v>
-      </c>
-      <c r="P40" t="n">
-        <v>57.91</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>16.63</v>
-      </c>
-      <c r="R40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61411,50 +59597,19 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>PPE, respirators, safety equipment</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E41" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
       </c>
       <c r="G41" t="n">
-        <v>221443.74</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H41" t="n">
-        <v>7</v>
+        <v>2.07</v>
       </c>
       <c r="I41" t="n">
-        <v>31634.82</v>
-      </c>
-      <c r="J41" t="n">
-        <v>25</v>
-      </c>
-      <c r="K41" t="n">
-        <v>51.57</v>
-      </c>
-      <c r="L41" t="n">
-        <v>57.14</v>
-      </c>
-      <c r="M41" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="N41" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="O41" t="n">
-        <v>2</v>
-      </c>
-      <c r="P41" t="n">
-        <v>85.40000000000001</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>2.07</v>
-      </c>
-      <c r="R41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61479,50 +59634,19 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Industrial PPE, gas detection</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E42" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
       </c>
       <c r="G42" t="n">
-        <v>344055.79</v>
+        <v>73.78</v>
       </c>
       <c r="H42" t="n">
-        <v>11</v>
+        <v>1.09</v>
       </c>
       <c r="I42" t="n">
-        <v>31277.8</v>
-      </c>
-      <c r="J42" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="K42" t="n">
-        <v>41.18</v>
-      </c>
-      <c r="L42" t="n">
-        <v>81.81999999999999</v>
-      </c>
-      <c r="M42" t="n">
-        <v>90.91</v>
-      </c>
-      <c r="N42" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="O42" t="n">
-        <v>2</v>
-      </c>
-      <c r="P42" t="n">
-        <v>73.78</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="R42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -61547,50 +59671,19 @@
           <t>Safety Equipment</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Local PPE distribution</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E43" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="F43" t="n">
+        <v>4</v>
       </c>
       <c r="G43" t="n">
-        <v>73346.89999999999</v>
+        <v>54.45</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>6.23</v>
       </c>
       <c r="I43" t="n">
-        <v>73346.89999999999</v>
-      </c>
-      <c r="J43" t="n">
-        <v>12</v>
-      </c>
-      <c r="K43" t="n">
-        <v>31</v>
-      </c>
-      <c r="L43" t="n">
-        <v>100</v>
-      </c>
-      <c r="M43" t="n">
-        <v>100</v>
-      </c>
-      <c r="N43" t="n">
-        <v>3.06</v>
-      </c>
-      <c r="O43" t="n">
-        <v>4</v>
-      </c>
-      <c r="P43" t="n">
-        <v>54.45</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>6.23</v>
-      </c>
-      <c r="R43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -61615,50 +59708,19 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Electrical systems, automation</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Core</t>
-        </is>
+      <c r="E44" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>9874558.890000001</v>
+        <v>85.73999999999999</v>
       </c>
       <c r="H44" t="n">
-        <v>31</v>
+        <v>1.56</v>
       </c>
       <c r="I44" t="n">
-        <v>318534.16</v>
-      </c>
-      <c r="J44" t="n">
-        <v>21.29</v>
-      </c>
-      <c r="K44" t="n">
-        <v>42.52</v>
-      </c>
-      <c r="L44" t="n">
-        <v>87.09999999999999</v>
-      </c>
-      <c r="M44" t="n">
-        <v>80.65000000000001</v>
-      </c>
-      <c r="N44" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="O44" t="n">
-        <v>0</v>
-      </c>
-      <c r="P44" t="n">
-        <v>85.73999999999999</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>1.56</v>
-      </c>
-      <c r="R44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61683,50 +59745,19 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Power distribution equipment</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E45" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
       </c>
       <c r="G45" t="n">
-        <v>1602186.6</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="H45" t="n">
-        <v>6</v>
+        <v>1.33</v>
       </c>
       <c r="I45" t="n">
-        <v>267031.1</v>
-      </c>
-      <c r="J45" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="K45" t="n">
-        <v>36.83</v>
-      </c>
-      <c r="L45" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="M45" t="n">
-        <v>100</v>
-      </c>
-      <c r="N45" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="O45" t="n">
-        <v>1</v>
-      </c>
-      <c r="P45" t="n">
-        <v>79.90000000000001</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="R45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61751,50 +59782,19 @@
           <t>Electrical &amp; Power</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Industrial automation, drives</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E46" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>2035290.13</v>
+        <v>88.38</v>
       </c>
       <c r="H46" t="n">
-        <v>9</v>
+        <v>0.95</v>
       </c>
       <c r="I46" t="n">
-        <v>226143.35</v>
-      </c>
-      <c r="J46" t="n">
-        <v>21.67</v>
-      </c>
-      <c r="K46" t="n">
-        <v>46.33</v>
-      </c>
-      <c r="L46" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="M46" t="n">
-        <v>66.67</v>
-      </c>
-      <c r="N46" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="O46" t="n">
-        <v>1</v>
-      </c>
-      <c r="P46" t="n">
-        <v>88.38</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61819,50 +59819,19 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Steel plates, structural steel</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E47" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="F47" t="n">
+        <v>3</v>
       </c>
       <c r="G47" t="n">
-        <v>893529.54</v>
+        <v>68.66</v>
       </c>
       <c r="H47" t="n">
-        <v>15</v>
+        <v>1.62</v>
       </c>
       <c r="I47" t="n">
-        <v>59568.64</v>
-      </c>
-      <c r="J47" t="n">
-        <v>10.87</v>
-      </c>
-      <c r="K47" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="L47" t="n">
-        <v>93.33</v>
-      </c>
-      <c r="M47" t="n">
-        <v>93.33</v>
-      </c>
-      <c r="N47" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="O47" t="n">
-        <v>3</v>
-      </c>
-      <c r="P47" t="n">
-        <v>68.66</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="R47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61887,50 +59856,19 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Steel products</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E48" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2</v>
       </c>
       <c r="G48" t="n">
-        <v>891500</v>
+        <v>68</v>
       </c>
       <c r="H48" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I48" t="n">
-        <v>127357.14</v>
-      </c>
-      <c r="J48" t="n">
-        <v>14.29</v>
-      </c>
-      <c r="K48" t="n">
-        <v>43.71</v>
-      </c>
-      <c r="L48" t="n">
-        <v>71.43000000000001</v>
-      </c>
-      <c r="M48" t="n">
-        <v>85.70999999999999</v>
-      </c>
-      <c r="N48" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="O48" t="n">
-        <v>2</v>
-      </c>
-      <c r="P48" t="n">
-        <v>68</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>4</v>
-      </c>
-      <c r="R48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61955,50 +59893,19 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Steel fabrication</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E49" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
       </c>
       <c r="G49" t="n">
-        <v>309528.45</v>
+        <v>81.64</v>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>4.49</v>
       </c>
       <c r="I49" t="n">
-        <v>77382.11</v>
-      </c>
-      <c r="J49" t="n">
-        <v>10.75</v>
-      </c>
-      <c r="K49" t="n">
-        <v>39</v>
-      </c>
-      <c r="L49" t="n">
-        <v>100</v>
-      </c>
-      <c r="M49" t="n">
-        <v>100</v>
-      </c>
-      <c r="N49" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="O49" t="n">
-        <v>4</v>
-      </c>
-      <c r="P49" t="n">
-        <v>81.64</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>4.49</v>
-      </c>
-      <c r="R49" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62023,50 +59930,19 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Local fabrication services</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E50" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F50" t="n">
+        <v>6</v>
       </c>
       <c r="G50" t="n">
-        <v>233377.11</v>
+        <v>57.59</v>
       </c>
       <c r="H50" t="n">
-        <v>3</v>
+        <v>2.3</v>
       </c>
       <c r="I50" t="n">
-        <v>77792.37</v>
-      </c>
-      <c r="J50" t="n">
-        <v>10</v>
-      </c>
-      <c r="K50" t="n">
-        <v>47.33</v>
-      </c>
-      <c r="L50" t="n">
-        <v>100</v>
-      </c>
-      <c r="M50" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="N50" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="O50" t="n">
-        <v>6</v>
-      </c>
-      <c r="P50" t="n">
-        <v>57.59</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="R50" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62091,50 +59967,19 @@
           <t>Local Steel</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Welding and fabrication</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E51" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2</v>
       </c>
       <c r="G51" t="n">
-        <v>456471.37</v>
+        <v>47.67</v>
       </c>
       <c r="H51" t="n">
-        <v>6</v>
+        <v>5.81</v>
       </c>
       <c r="I51" t="n">
-        <v>76078.56</v>
-      </c>
-      <c r="J51" t="n">
-        <v>8.17</v>
-      </c>
-      <c r="K51" t="n">
-        <v>31.67</v>
-      </c>
-      <c r="L51" t="n">
-        <v>100</v>
-      </c>
-      <c r="M51" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="N51" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="O51" t="n">
-        <v>2</v>
-      </c>
-      <c r="P51" t="n">
-        <v>47.67</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>5.81</v>
-      </c>
-      <c r="R51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62159,50 +60004,19 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Heavy hauling, logistics services</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>Established</t>
-        </is>
+      <c r="E52" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="F52" t="n">
+        <v>3</v>
       </c>
       <c r="G52" t="n">
-        <v>456430.44</v>
+        <v>60.96</v>
       </c>
       <c r="H52" t="n">
-        <v>5</v>
+        <v>0.95</v>
       </c>
       <c r="I52" t="n">
-        <v>91286.09</v>
-      </c>
-      <c r="J52" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="K52" t="n">
-        <v>35.8</v>
-      </c>
-      <c r="L52" t="n">
-        <v>100</v>
-      </c>
-      <c r="M52" t="n">
-        <v>100</v>
-      </c>
-      <c r="N52" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="O52" t="n">
-        <v>3</v>
-      </c>
-      <c r="P52" t="n">
-        <v>60.96</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="R52" t="n">
         <v>1</v>
       </c>
     </row>
@@ -62227,50 +60041,19 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Coal shipping services</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E53" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="F53" t="n">
+        <v>4</v>
       </c>
       <c r="G53" t="n">
-        <v>479055.53</v>
+        <v>19.67</v>
       </c>
       <c r="H53" t="n">
-        <v>6</v>
+        <v>2.23</v>
       </c>
       <c r="I53" t="n">
-        <v>79842.59</v>
-      </c>
-      <c r="J53" t="n">
-        <v>13.17</v>
-      </c>
-      <c r="K53" t="n">
-        <v>30.17</v>
-      </c>
-      <c r="L53" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="M53" t="n">
-        <v>100</v>
-      </c>
-      <c r="N53" t="n">
-        <v>6.33</v>
-      </c>
-      <c r="O53" t="n">
-        <v>4</v>
-      </c>
-      <c r="P53" t="n">
-        <v>19.67</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="R53" t="n">
         <v>1</v>
       </c>
     </row>
@@ -62295,50 +60078,19 @@
           <t>Logistics &amp; Transport</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Land transportation</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E54" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F54" t="n">
+        <v>3</v>
       </c>
       <c r="G54" t="n">
-        <v>145604.12</v>
+        <v>87.14</v>
       </c>
       <c r="H54" t="n">
-        <v>2</v>
+        <v>1.78</v>
       </c>
       <c r="I54" t="n">
-        <v>72802.06</v>
-      </c>
-      <c r="J54" t="n">
-        <v>8</v>
-      </c>
-      <c r="K54" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="L54" t="n">
-        <v>100</v>
-      </c>
-      <c r="M54" t="n">
-        <v>100</v>
-      </c>
-      <c r="N54" t="n">
-        <v>2.04</v>
-      </c>
-      <c r="O54" t="n">
-        <v>3</v>
-      </c>
-      <c r="P54" t="n">
-        <v>87.14</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="R54" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62363,50 +60115,19 @@
           <t>Spare Parts &amp; Components</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Genuine spare parts distribution</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E55" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F55" t="n">
+        <v>2</v>
       </c>
       <c r="G55" t="n">
-        <v>262321.84</v>
+        <v>76.73999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="I55" t="n">
-        <v>262321.84</v>
-      </c>
-      <c r="J55" t="n">
-        <v>8</v>
-      </c>
-      <c r="K55" t="n">
-        <v>29</v>
-      </c>
-      <c r="L55" t="n">
-        <v>100</v>
-      </c>
-      <c r="M55" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" t="n">
-        <v>3.45</v>
-      </c>
-      <c r="O55" t="n">
-        <v>2</v>
-      </c>
-      <c r="P55" t="n">
-        <v>76.73999999999999</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>8.470000000000001</v>
-      </c>
-      <c r="R55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62431,50 +60152,19 @@
           <t>Spare Parts &amp; Components</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Aftermarket spare parts</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
+      <c r="E56" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>7</v>
       </c>
       <c r="G56" t="n">
-        <v>322104.23</v>
+        <v>68.08</v>
       </c>
       <c r="H56" t="n">
-        <v>2</v>
+        <v>3.54</v>
       </c>
       <c r="I56" t="n">
-        <v>161052.12</v>
-      </c>
-      <c r="J56" t="n">
-        <v>12</v>
-      </c>
-      <c r="K56" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="L56" t="n">
-        <v>50</v>
-      </c>
-      <c r="M56" t="n">
-        <v>100</v>
-      </c>
-      <c r="N56" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="O56" t="n">
-        <v>7</v>
-      </c>
-      <c r="P56" t="n">
-        <v>68.08</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>3.54</v>
-      </c>
-      <c r="R56" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>